<commit_message>
Leads: 2026-10-24 12:49 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,62 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Thomas E Clark Inc</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>thomaseclark.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.thomaseclark.com/areas-we-serve/germantown-md/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>chris@thomaseclark.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(301) 608-0550</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Germantown MD</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>heating and cooling company Germantown MD</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-24 18:44 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://www.thomaseclark.com/areas-we-serve/germantown-md/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>chris@thomaseclark.com</t>
@@ -614,6 +613,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pioneer Plumbing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pioneerplumbingidaho.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://pioneerplumbingidaho.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Reviews Gallery</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>letstalk@pioneerplumbingidaho.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(208) 540-9444</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>emergency plumber Boise ID</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-24 18:48 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Roofing Company in Charlotte, NC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>grierroofing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://grierroofing.com/areas-we-serve/roofing-company-charlotte-nc/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>South Carolina</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>office@grierroofing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>864.578.0968</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Charlotte NC</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>residential roofing company Charlotte NC</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-24 18:50 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Better Builders Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>betterbuildersroofing.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://betterbuildersroofing.com/roofing/roof-replacement/aurora</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Marine Corps</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>mybetterbuilders@outlook.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(303) 319-5727</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roof replacement Aurora CO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-24 18:51 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,126 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Phoenix &amp; Scottsdale | Same-Day Clog Removal | Drain Surgeons</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>drainsurgeonsaz.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://drainsurgeonsaz.com/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@drainsrgn.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>480-696-1777</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>drain cleaning service Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wyman Plumbing &amp; Mechanical</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>wyman-services.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.wyman-services.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Drain Audit</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>office@wyman-services.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(623) 236-2097</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>drain cleaning service Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-24 18:59 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sullys Heating and Air</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>sullysheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://sullysheatingandair.com/orem/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Service Serving</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>sullysheatingandair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(801) 599-9007</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>air conditioning repair Orem UT</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-24 19:03 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,118 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Expert HVAC Services | Thomas J. Fannon &amp; Sons | Alexandria, VA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>tjfannon.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.tjfannon.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>jakefannon@tjfannon.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(703) 549-5700</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Alexandria VA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>heating and cooling company Alexandria VA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Metal Roofing Installation in Danbury</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>danbury-ct.americaroofingco.org</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://danbury-ct.americaroofingco.org/metal-roofing-installation.html</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@americaroofingco.org</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(855) 946-2064</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Danbury CT</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Danbury CT</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-24 19:05 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -999,7 +999,6 @@
           <t>https://www.tjfannon.com/</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>jakefannon@tjfannon.com</t>
@@ -1055,7 +1054,6 @@
           <t>https://danbury-ct.americaroofingco.org/metal-roofing-installation.html</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>info@americaroofingco.org</t>
@@ -1085,6 +1083,66 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Orlando Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>orlando-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://orlando-metal-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@orlando-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(321) 325-4217</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Orlando FL</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-24 19:08 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-24.xlsx
+++ b/output/leads_2026-10-24.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1148,6 +1148,66 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Comfort Airz Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>comfortairz.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://comfortairz.com/clearwater-fl-ac-replacement/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>inquiries@comfortairz.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(888) 552-2479</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>AC installation Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>